<commit_message>
📝 docs (budget): update
</commit_message>
<xml_diff>
--- a/public/documents/budget_en.xlsx
+++ b/public/documents/budget_en.xlsx
@@ -1438,9 +1438,9 @@
         <f t="shared" ref="F14:F19" si="1">PRODUCT(D14:E14)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="49">
-        <f t="shared" ref="G14:G15" si="2">PRODUCT(F8:F14)</f>
-        <v>0</v>
+      <c r="G14" s="49" t="str">
+        <f>PRODUCT(F14/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
@@ -1455,9 +1455,9 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G15" s="49">
-        <f t="shared" si="2"/>
-        <v>0</v>
+      <c r="G15" s="49" t="str">
+        <f>PRODUCT(F15/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
@@ -1472,9 +1472,9 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G16" s="49">
-        <f t="shared" ref="G16:G17" si="3">PRODUCT(F11:F17)</f>
-        <v>0</v>
+      <c r="G16" s="49" t="str">
+        <f>PRODUCT(F17/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
@@ -1489,9 +1489,9 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G17" s="49">
-        <f t="shared" si="3"/>
-        <v>0</v>
+      <c r="G17" s="49" t="str">
+        <f>PRODUCT(F18/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
@@ -1506,9 +1506,9 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G18" s="49">
-        <f t="shared" ref="G18:G19" si="4">PRODUCT(F12:F18)</f>
-        <v>0</v>
+      <c r="G18" s="49" t="str">
+        <f>PRODUCT(F18/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="19" ht="14.25" customHeight="1">
@@ -1523,9 +1523,9 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G19" s="49">
-        <f t="shared" si="4"/>
-        <v>0</v>
+      <c r="G19" s="49" t="str">
+        <f>PRODUCT(F19/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
@@ -1537,12 +1537,12 @@
       <c r="D20" s="58"/>
       <c r="E20" s="59"/>
       <c r="F20" s="59">
-        <f t="shared" ref="F20:G20" si="5">SUM(F14:F19)</f>
+        <f t="shared" ref="F20:G20" si="2">SUM(F14:F19)</f>
         <v>0</v>
       </c>
-      <c r="G20" s="60">
-        <f t="shared" si="5"/>
-        <v>0</v>
+      <c r="G20" s="60" t="str">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
       </c>
       <c r="H20" s="61"/>
       <c r="I20" s="61"/>
@@ -1585,12 +1585,12 @@
       <c r="D22" s="70"/>
       <c r="E22" s="71"/>
       <c r="F22" s="48">
-        <f t="shared" ref="F22:F26" si="6">PRODUCT(D22:E22)</f>
+        <f t="shared" ref="F22:F26" si="3">PRODUCT(D22:E22)</f>
         <v>0</v>
       </c>
-      <c r="G22" s="49">
-        <f t="shared" ref="G22:G26" si="7">PRODUCT(F17:F23)</f>
-        <v>0</v>
+      <c r="G22" s="49" t="str">
+        <f>PRODUCT(F22/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="23" ht="14.25" customHeight="1">
@@ -1602,12 +1602,12 @@
       <c r="D23" s="70"/>
       <c r="E23" s="71"/>
       <c r="F23" s="48">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G23" s="49">
-        <f t="shared" si="7"/>
-        <v>0</v>
+      <c r="G23" s="49" t="str">
+        <f>PRODUCT(F23/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="24" ht="14.25" customHeight="1">
@@ -1619,12 +1619,12 @@
       <c r="D24" s="70"/>
       <c r="E24" s="71"/>
       <c r="F24" s="48">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G24" s="49">
-        <f t="shared" si="7"/>
-        <v>0</v>
+      <c r="G24" s="49" t="str">
+        <f>PRODUCT(F24/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="25" ht="14.25" customHeight="1">
@@ -1636,12 +1636,12 @@
       <c r="D25" s="70"/>
       <c r="E25" s="71"/>
       <c r="F25" s="48">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G25" s="49">
-        <f t="shared" si="7"/>
-        <v>0</v>
+      <c r="G25" s="49" t="str">
+        <f>PRODUCT(F25/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="26" ht="14.25" customHeight="1">
@@ -1653,12 +1653,12 @@
       <c r="D26" s="73"/>
       <c r="E26" s="74"/>
       <c r="F26" s="48">
-        <f t="shared" si="6"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G26" s="49">
-        <f t="shared" si="7"/>
-        <v>0</v>
+      <c r="G26" s="49" t="str">
+        <f>PRODUCT(F26/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="27" ht="14.25" customHeight="1">
@@ -1673,9 +1673,9 @@
         <f>SUM(F22:F25)</f>
         <v>0</v>
       </c>
-      <c r="G27" s="75">
+      <c r="G27" s="75" t="str">
         <f>SUM(G22:G26)</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="H27" s="61"/>
       <c r="I27" s="61"/>
@@ -1736,12 +1736,12 @@
       <c r="D29" s="80"/>
       <c r="E29" s="54"/>
       <c r="F29" s="48">
-        <f t="shared" ref="F29:F33" si="8">PRODUCT(D29:E29)</f>
+        <f t="shared" ref="F29:F33" si="4">PRODUCT(D29:E29)</f>
         <v>0</v>
       </c>
-      <c r="G29" s="49">
-        <f t="shared" ref="G29:G33" si="9">PRODUCT(F24:F30)</f>
-        <v>0</v>
+      <c r="G29" s="49" t="str">
+        <f>PRODUCT(F29/F8)</f>
+        <v>#DIV/0!</v>
       </c>
       <c r="H29" s="78"/>
       <c r="I29" s="78"/>
@@ -1771,12 +1771,12 @@
       <c r="D30" s="80"/>
       <c r="E30" s="54"/>
       <c r="F30" s="48">
-        <f t="shared" si="8"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G30" s="49">
-        <f t="shared" si="9"/>
-        <v>0</v>
+      <c r="G30" s="49" t="str">
+        <f>PRODUCT(F30/F8)</f>
+        <v>#DIV/0!</v>
       </c>
       <c r="H30" s="78"/>
       <c r="I30" s="78"/>
@@ -1806,12 +1806,12 @@
       <c r="D31" s="80"/>
       <c r="E31" s="54"/>
       <c r="F31" s="48">
-        <f t="shared" si="8"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G31" s="49">
-        <f t="shared" si="9"/>
-        <v>0</v>
+      <c r="G31" s="49" t="str">
+        <f>PRODUCT(F31/F8)</f>
+        <v>#DIV/0!</v>
       </c>
       <c r="H31" s="78"/>
       <c r="I31" s="78"/>
@@ -1841,12 +1841,12 @@
       <c r="D32" s="80"/>
       <c r="E32" s="54"/>
       <c r="F32" s="48">
-        <f t="shared" si="8"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G32" s="49">
-        <f t="shared" si="9"/>
-        <v>0</v>
+      <c r="G32" s="49" t="str">
+        <f>PRODUCT(F32/F8)</f>
+        <v>#DIV/0!</v>
       </c>
       <c r="H32" s="78"/>
       <c r="I32" s="78"/>
@@ -1876,12 +1876,12 @@
       <c r="D33" s="80"/>
       <c r="E33" s="54"/>
       <c r="F33" s="48">
-        <f t="shared" si="8"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G33" s="49">
-        <f t="shared" si="9"/>
-        <v>0</v>
+      <c r="G33" s="49" t="str">
+        <f>PRODUCT(F33/F8)</f>
+        <v>#DIV/0!</v>
       </c>
       <c r="H33" s="78"/>
       <c r="I33" s="78"/>
@@ -1911,12 +1911,12 @@
       <c r="D34" s="86"/>
       <c r="E34" s="87"/>
       <c r="F34" s="88">
-        <f t="shared" ref="F34:G34" si="10">SUM(F29:F33)</f>
+        <f t="shared" ref="F34:G34" si="5">SUM(F29:F33)</f>
         <v>0</v>
       </c>
-      <c r="G34" s="60">
-        <f t="shared" si="10"/>
-        <v>0</v>
+      <c r="G34" s="60" t="str">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
       </c>
       <c r="H34" s="78"/>
       <c r="I34" s="78"/>
@@ -1986,12 +1986,12 @@
       <c r="D37" s="101"/>
       <c r="E37" s="99"/>
       <c r="F37" s="48">
-        <f t="shared" ref="F37:F43" si="11">PRODUCT(D37:E37)</f>
+        <f t="shared" ref="F37:F43" si="6">PRODUCT(D37:E37)</f>
         <v>0</v>
       </c>
-      <c r="G37" s="49">
-        <f t="shared" ref="G37:G43" si="12">PRODUCT(F32:F38)</f>
-        <v>0</v>
+      <c r="G37" s="49" t="str">
+        <f>PRODUCT(F37/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="38" ht="16.5" customHeight="1">
@@ -2003,12 +2003,12 @@
       <c r="D38" s="103"/>
       <c r="E38" s="99"/>
       <c r="F38" s="48">
-        <f t="shared" si="11"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G38" s="49">
-        <f t="shared" si="12"/>
-        <v>0</v>
+      <c r="G38" s="49" t="str">
+        <f>PRODUCT(F38/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="39" ht="16.5" customHeight="1">
@@ -2020,12 +2020,12 @@
       <c r="D39" s="103"/>
       <c r="E39" s="104"/>
       <c r="F39" s="48">
-        <f t="shared" si="11"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G39" s="49">
-        <f t="shared" si="12"/>
-        <v>0</v>
+      <c r="G39" s="49" t="str">
+        <f>PRODUCT(F39/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="40" ht="16.5" customHeight="1">
@@ -2037,12 +2037,12 @@
       <c r="D40" s="103"/>
       <c r="E40" s="104"/>
       <c r="F40" s="48">
-        <f t="shared" si="11"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G40" s="49">
-        <f t="shared" si="12"/>
-        <v>0</v>
+      <c r="G40" s="49" t="str">
+        <f>PRODUCT(F40/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="41" ht="16.5" customHeight="1">
@@ -2054,12 +2054,12 @@
       <c r="D41" s="103"/>
       <c r="E41" s="99"/>
       <c r="F41" s="48">
-        <f t="shared" si="11"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G41" s="49">
-        <f t="shared" si="12"/>
-        <v>0</v>
+      <c r="G41" s="49" t="str">
+        <f>PRODUCT(F41/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="42" ht="16.5" customHeight="1">
@@ -2070,12 +2070,12 @@
       <c r="D42" s="2"/>
       <c r="E42" s="105"/>
       <c r="F42" s="48">
-        <f t="shared" si="11"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G42" s="49">
-        <f t="shared" si="12"/>
-        <v>0</v>
+      <c r="G42" s="49" t="str">
+        <f>PRODUCT(F42/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="43" ht="16.5" customHeight="1">
@@ -2087,12 +2087,12 @@
       <c r="D43" s="107"/>
       <c r="E43" s="108"/>
       <c r="F43" s="48">
-        <f t="shared" si="11"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G43" s="49">
-        <f t="shared" si="12"/>
-        <v>0</v>
+      <c r="G43" s="49" t="str">
+        <f>PRODUCT(F43/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="44" ht="16.5" customHeight="1">
@@ -2107,9 +2107,9 @@
         <f>SUM(F37:F39)</f>
         <v>0</v>
       </c>
-      <c r="G44" s="60">
+      <c r="G44" s="60" t="str">
         <f>SUM(G37:G43)</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="45" ht="16.5" customHeight="1">
@@ -2135,9 +2135,9 @@
         <f>SUM(F44,F34,F27,F20,)</f>
         <v>0</v>
       </c>
-      <c r="G46" s="60">
-        <f>PRODUCT(F8:F46)</f>
-        <v>0</v>
+      <c r="G46" s="60" t="str">
+        <f>PRODUCT(F46/F8)</f>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="47" ht="27.75" customHeight="1">
@@ -2151,9 +2151,9 @@
       <c r="D47" s="128"/>
       <c r="E47" s="128"/>
       <c r="F47" s="128"/>
-      <c r="G47" s="129">
+      <c r="G47" s="129" t="str">
         <f>SUM(G20+G27+G34+G44)</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="H47" s="130"/>
       <c r="I47" s="130"/>
@@ -5868,19 +5868,19 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="C10:C12"/>
     <mergeCell ref="D10:D12"/>
-    <mergeCell ref="B47:F47"/>
     <mergeCell ref="E10:F10"/>
-    <mergeCell ref="G10:G12"/>
     <mergeCell ref="E11:E12"/>
     <mergeCell ref="F11:F12"/>
+    <mergeCell ref="B47:F47"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="B6:G6"/>
     <mergeCell ref="B7:D8"/>
     <mergeCell ref="E7:G7"/>
     <mergeCell ref="A10:A12"/>
     <mergeCell ref="B10:B12"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="G10:G12"/>
   </mergeCells>
   <dataValidations>
     <dataValidation type="decimal" allowBlank="1" showDropDown="1" showInputMessage="1" prompt="Saisissez un nombre compris entre 1 et 10000" sqref="F8">

</xml_diff>